<commit_message>
Integrate AI tags into the pipeline
</commit_message>
<xml_diff>
--- a/tests/anki_addons_dataset/exporter/xlsx/exp_data.xlsx
+++ b/tests/anki_addons_dataset/exporter/xlsx/exp_data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Addons" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Addons!$A$3:$V$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Addons!$A$3:$W$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -113,12 +113,25 @@
         </r>
       </text>
     </comment>
+    <comment ref="W3" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Tags chosen by an AI model from a fixed vocabulary, based on the AnkiWeb description and the GitHub README. Blank = not generated yet.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="40">
   <si>
     <t>Anki Addons Dataset</t>
   </si>
@@ -204,6 +217,9 @@
     <t>Summary</t>
   </si>
   <si>
+    <t>Tags</t>
+  </si>
+  <si>
     <t>NoteSize</t>
   </si>
   <si>
@@ -223,6 +239,9 @@
   </si>
   <si>
     <t>Shows the size of the collection and of individual notes.</t>
+  </si>
+  <si>
+    <t>statistics</t>
   </si>
   <si>
     <t>2023-09-10</t>
@@ -610,7 +629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -631,9 +650,10 @@
     <col min="20" max="20" width="8.7109375" customWidth="1"/>
     <col min="21" max="21" width="13.7109375" customWidth="1"/>
     <col min="22" max="22" width="80.7109375" customWidth="1"/>
+    <col min="23" max="23" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22">
+    <row r="1" spans="1:23">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -657,7 +677,7 @@
       </c>
       <c r="N1" s="3"/>
     </row>
-    <row r="2" spans="1:22">
+    <row r="2" spans="1:23">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -688,8 +708,9 @@
       <c r="V2" s="4" t="s">
         <v>26</v>
       </c>
+      <c r="W2" s="4"/>
     </row>
-    <row r="3" spans="1:22">
+    <row r="3" spans="1:23">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
@@ -756,19 +777,22 @@
       <c r="V3" s="4" t="s">
         <v>27</v>
       </c>
+      <c r="W3" s="4" t="s">
+        <v>28</v>
+      </c>
     </row>
-    <row r="4" spans="1:22">
+    <row r="4" spans="1:23">
       <c r="A4">
         <v>1188705668</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -783,34 +807,34 @@
         <v>0</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="J4" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>32</v>
-      </c>
-      <c r="K4" t="s">
-        <v>33</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>31</v>
       </c>
       <c r="M4">
         <v>42</v>
       </c>
       <c r="N4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P4">
         <v>3</v>
       </c>
       <c r="Q4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="S4">
         <v>5</v>
@@ -819,15 +843,18 @@
         <v>7</v>
       </c>
       <c r="U4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="V4" t="s">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="W4" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:V3"/>
-  <mergeCells count="8">
+  <autoFilter ref="A3:W3"/>
+  <mergeCells count="9">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:F1"/>
@@ -836,6 +863,7 @@
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="L2:N2"/>
     <mergeCell ref="O2:U2"/>
+    <mergeCell ref="V2:W2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="I4" r:id="rId1"/>

</xml_diff>